<commit_message>
incorrect values condensed, fixes to final submission, all other changes before cleaning up landing page
</commit_message>
<xml_diff>
--- a/data/oecd_comments.xlsx
+++ b/data/oecd_comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kate/OneDrive/WISE/Data request portal/data-request-portal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625110E6-58D8-CD4A-99DB-148E0D6E8AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38A4FF6-5C29-4C42-A02E-A52BE753AEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="75">
   <si>
     <t>ref_area</t>
   </si>
@@ -253,6 +253,15 @@
   </si>
   <si>
     <t>FIN</t>
+  </si>
+  <si>
+    <t>PER</t>
+  </si>
+  <si>
+    <t>Thank you for letting us know about this indicator. More information on the question(s) phrasing behind this data is required before it may be validated and added to the Well-being Database.</t>
+  </si>
+  <si>
+    <t>More information on how a depressive episode is defined and how the data is collected is required</t>
   </si>
 </sst>
 </file>
@@ -302,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -312,6 +321,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -610,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="65.5" style="1" customWidth="1"/>
@@ -1596,7 +1608,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>31</v>
       </c>
@@ -1607,7 +1619,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>38</v>
       </c>
@@ -1618,7 +1630,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>38</v>
       </c>
@@ -1629,7 +1641,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>66</v>
       </c>
@@ -1640,7 +1652,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>45</v>
       </c>
@@ -1651,7 +1663,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>47</v>
       </c>
@@ -1662,7 +1674,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>47</v>
       </c>
@@ -1673,7 +1685,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>47</v>
       </c>
@@ -1684,7 +1696,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>47</v>
       </c>
@@ -1693,6 +1705,90 @@
       </c>
       <c r="C89" s="1" t="s">
         <v>57</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>72</v>
+      </c>
+      <c r="B90" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>72</v>
+      </c>
+      <c r="B91" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>72</v>
+      </c>
+      <c r="B92" t="s">
+        <v>35</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>72</v>
+      </c>
+      <c r="B93" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>72</v>
+      </c>
+      <c r="B94" t="s">
+        <v>14</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>72</v>
+      </c>
+      <c r="B95" t="s">
+        <v>16</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stable storage, final bug fixes
</commit_message>
<xml_diff>
--- a/data/oecd_comments.xlsx
+++ b/data/oecd_comments.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kate/OneDrive/WISE/Data request portal/data-request-portal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EABEBE21-F67D-5B43-8E9C-89BF846BF92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD98B9C-7EB0-984D-87E9-422468EDDB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$C$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$92</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="81">
   <si>
     <t>ref_area</t>
   </si>
@@ -153,9 +153,6 @@
     <t>NOR</t>
   </si>
   <si>
-    <t>POL</t>
-  </si>
-  <si>
     <t>KOR</t>
   </si>
   <si>
@@ -198,9 +195,6 @@
     <t>5-point scale rather than 6-point scale used by the OECD</t>
   </si>
   <si>
-    <t>2-point scale rather than 5-point scale used by the OECD</t>
-  </si>
-  <si>
     <t>Thank you for submitting data in a previous request. However the percentages should be in percentage of the subgroup (so number of women who voted / percentage of total population of women) not the entire population. Would it be possible to provide data by subgroup?</t>
   </si>
   <si>
@@ -213,18 +207,9 @@
     <t>Thank you for letting us know about this indicator. Unfortunately, we are unable to publish it in the Well-being Database because it does not match the OECD harmonised response format. We would still be happy to receive any updated submissions on it for record-keeping, where it remains available for future reference and analysis.</t>
   </si>
   <si>
-    <t>5-point scale rather than 6-point scale used by the OECD. EU-SILC data is currently being used.</t>
-  </si>
-  <si>
-    <t>AUT</t>
-  </si>
-  <si>
     <t>PHQ comparison pending</t>
   </si>
   <si>
-    <t>4-point scale rather than 5-point used by the OECD</t>
-  </si>
-  <si>
     <t>Measure of satisfaction rather than distance to park</t>
   </si>
   <si>
@@ -262,6 +247,39 @@
   </si>
   <si>
     <t>Time use tables were not completed so validation of values was not possible. Also, value corrupted due to input as a time value (11:35 PM), please recalculate.</t>
+  </si>
+  <si>
+    <t>Time use tables were not completed so validation of values was not possible. Also, value corrupted due to input as a time value (37:16), please recalculate.</t>
+  </si>
+  <si>
+    <t>Thank you for submitting data in a previous request. Unfortunately we were not able to harmonize it with the other data in the Well-being Database either due to Time Use tables not being filled out, incomplete or with errors in submission. Please fill in the Time Use Tables on the Time Use Submission tab so we may validate the data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The previous Time Use Data Submission could not be validated because the sub-values in the table did not correspond with the total values submitted by each time use category. </t>
+  </si>
+  <si>
+    <t>No Time Use table was filled out.</t>
+  </si>
+  <si>
+    <t>Data does not come from a Time Use survey.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time use tables were not completed so validation of values was not possible. </t>
+  </si>
+  <si>
+    <t>Following previous correspondance with OECD about categorisation of unpaid work, please double check these values to make sure they are consistent with changes.</t>
+  </si>
+  <si>
+    <t>Categorisation of activities did not align with those of the OECD data, please align and re-submit.</t>
+  </si>
+  <si>
+    <t>Following previous correspondance with OECD about harominsation of Time Use tables, please recompute these values accordingly.</t>
+  </si>
+  <si>
+    <t>Data will be collected directly from source so no need for submission</t>
+  </si>
+  <si>
+    <t>Question phrasing is different from OECD's source. Also, 4-point scale rather than 6-point used by the OECD.</t>
   </si>
 </sst>
 </file>
@@ -622,11 +640,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D95"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="65.5" style="1" customWidth="1"/>
     <col min="4" max="4" width="27.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -643,7 +663,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -651,13 +671,13 @@
         <v>5</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -665,10 +685,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -676,10 +696,13 @@
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -687,10 +710,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -698,10 +721,10 @@
         <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -709,10 +732,13 @@
         <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -720,1085 +746,1110 @@
         <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="C12" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>68</v>
-      </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>50</v>
+        <v>5</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>55</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
-        <v>19</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="96" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>21</v>
       </c>
       <c r="B36" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" t="s">
         <v>6</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>21</v>
-      </c>
-      <c r="B37" t="s">
+      <c r="C37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>69</v>
-      </c>
-      <c r="B38" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>69</v>
-      </c>
-      <c r="B39" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>69</v>
-      </c>
-      <c r="B40" t="s">
-        <v>8</v>
-      </c>
       <c r="C40" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>57</v>
+        <v>33</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>33</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>18</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>57</v>
+        <v>14</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" t="s">
         <v>7</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>67</v>
-      </c>
-      <c r="B49" t="s">
-        <v>6</v>
-      </c>
       <c r="C49" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B50" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B51" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="B52" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>50</v>
+        <v>5</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>24</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>24</v>
       </c>
       <c r="B56" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>24</v>
       </c>
       <c r="B57" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B58" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B59" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B60" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B61" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B62" t="s">
-        <v>16</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B63" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B64" t="s">
-        <v>8</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B65" t="s">
-        <v>35</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B66" t="s">
-        <v>4</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>43</v>
+        <v>18</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B67" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B68" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="B69" t="s">
-        <v>5</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>27</v>
       </c>
       <c r="B70" t="s">
-        <v>4</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>27</v>
       </c>
       <c r="B71" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B72" t="s">
-        <v>19</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>57</v>
+        <v>16</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>37</v>
       </c>
       <c r="B73" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>37</v>
       </c>
       <c r="B74" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>37</v>
       </c>
       <c r="B75" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>37</v>
       </c>
       <c r="B76" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B77" t="s">
-        <v>10</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B78" t="s">
-        <v>5</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>57</v>
+        <v>9</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B79" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B80" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B81" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>38</v>
       </c>
       <c r="B82" t="s">
+        <v>19</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>24</v>
+      </c>
+      <c r="B83" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>46</v>
+      </c>
+      <c r="B84" t="s">
         <v>6</v>
       </c>
-      <c r="C82" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>38</v>
-      </c>
-      <c r="B83" t="s">
+      <c r="C84" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>46</v>
+      </c>
+      <c r="B85" t="s">
         <v>8</v>
       </c>
-      <c r="C83" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>64</v>
-      </c>
-      <c r="B84" t="s">
+      <c r="C85" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>46</v>
+      </c>
+      <c r="B86" t="s">
+        <v>10</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>65</v>
+      </c>
+      <c r="B87" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>65</v>
+      </c>
+      <c r="B88" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>65</v>
+      </c>
+      <c r="B89" t="s">
         <v>16</v>
       </c>
-      <c r="C84" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="64" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>45</v>
-      </c>
-      <c r="B85" t="s">
+      <c r="C89" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>59</v>
+      </c>
+      <c r="B90" t="s">
+        <v>16</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>44</v>
+      </c>
+      <c r="B91" t="s">
         <v>11</v>
       </c>
-      <c r="C85" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+      <c r="C91" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>46</v>
+      </c>
+      <c r="B92" t="s">
         <v>47</v>
       </c>
-      <c r="B86" t="s">
-        <v>48</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>47</v>
-      </c>
-      <c r="B87" t="s">
-        <v>6</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>47</v>
-      </c>
-      <c r="B88" t="s">
-        <v>8</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>47</v>
-      </c>
-      <c r="B89" t="s">
-        <v>10</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>70</v>
-      </c>
-      <c r="B90" t="s">
-        <v>5</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>70</v>
-      </c>
-      <c r="B91" t="s">
-        <v>5</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>70</v>
-      </c>
-      <c r="B92" t="s">
-        <v>35</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>57</v>
+      <c r="C92" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="64" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>70</v>
-      </c>
-      <c r="B93" t="s">
-        <v>4</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>70</v>
-      </c>
-      <c r="B94" t="s">
-        <v>14</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="80" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>70</v>
-      </c>
-      <c r="B95" t="s">
-        <v>16</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D95" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C72" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C89">
-      <sortCondition ref="A1:A89"/>
+  <autoFilter xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" ref="A1:D92" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <x14:filter val="Thank you for letting us know about this indicator. Unfortunately, we are unable to publish it in the Well-being Database because it does not match the OECD harmonised response format. We would still be happy to receive any updated submissions on it for record-keeping, where it remains available for future reference and analysis."/>
+            <x14:filter val="Thank you for submitting this data. In the previous request, the country average was not included among the data shared, would you it be possible to update the values to include it?"/>
+          </mc:Choice>
+          <mc:Fallback>
+            <filter val="Thank you for submitting this data. In the previous request, the country average was not included among the data shared, would you it be possible to update the values to include it?"/>
+          </mc:Fallback>
+        </mc:AlternateContent>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters blank="1"/>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:D83">
+      <sortCondition ref="B1:B92"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C31">
-    <sortCondition ref="A1:A31"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C30">
+    <sortCondition ref="A1:A30"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
prefill previous responses + update comments
</commit_message>
<xml_diff>
--- a/data/oecd_comments.xlsx
+++ b/data/oecd_comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kate/OneDrive/WISE/Data request portal/data-request-portal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0986939A-D774-214A-9EA2-9B7CF22F38CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BFAFAF-1DF3-2D47-8312-5022411BF0D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$115</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="113">
   <si>
     <t>ref_area</t>
   </si>
@@ -189,9 +189,6 @@
     <t>Categorisation of activities did not align with those of the OECD data, please align and re-submit.</t>
   </si>
   <si>
-    <t>Following previous correspondance with OECD about harominsation of Time Use tables, please recompute these values accordingly.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Question phrasing is different from OECD's source. </t>
   </si>
   <si>
@@ -367,6 +364,18 @@
   </si>
   <si>
     <t>Please provide a response format (is it yes or no?). Also, no country average was provided.</t>
+  </si>
+  <si>
+    <t>Time use tables were not completed, please fill out the Time Use Submission tab so this indicator may be validated. In addition, unit is not correct, please recalculate as total minutes per day. Finally, would it be possible to also calculate values for 2022?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Following previous correspondance with OECD about harominsation of Time Use tables, please recompute these values accordingly. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Following previous correspondance with OECD about harominsation of Time Use tables, please recompute these values accordingly. Values were reported as 2016 and 2021, adjusted 2016 to 2014 and 2021 to 2019, please confirm change. </t>
+  </si>
+  <si>
+    <t>Following previous correspondance with OECD about harominsation of Time Use tables, please recompute these values accordingly. Also please review 2014 values and education values for 2019 for harmony with unit measure of hours per week.</t>
   </si>
 </sst>
 </file>
@@ -728,7 +737,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="65.5" style="1" customWidth="1"/>
@@ -758,10 +767,10 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -775,12 +784,12 @@
         <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
         <v>39</v>
@@ -803,7 +812,7 @@
         <v>41</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -817,7 +826,7 @@
         <v>41</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -828,7 +837,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -842,12 +851,12 @@
         <v>41</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -870,7 +879,7 @@
         <v>41</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
@@ -884,7 +893,7 @@
         <v>41</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -909,7 +918,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -928,7 +937,7 @@
     </row>
     <row r="15" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
@@ -951,7 +960,7 @@
         <v>41</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -965,7 +974,7 @@
         <v>41</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -990,10 +999,10 @@
         <v>15</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1007,12 +1016,12 @@
         <v>41</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="128" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
         <v>15</v>
@@ -1021,7 +1030,7 @@
         <v>41</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="128" hidden="1" x14ac:dyDescent="0.2">
@@ -1035,7 +1044,7 @@
         <v>41</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1046,10 +1055,10 @@
         <v>23</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1063,7 +1072,7 @@
         <v>41</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1074,10 +1083,10 @@
         <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1088,7 +1097,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1113,24 +1122,24 @@
         <v>6</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
@@ -1141,24 +1150,24 @@
         <v>6</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B31" t="s">
         <v>6</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
@@ -1169,10 +1178,10 @@
         <v>6</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="128" hidden="1" x14ac:dyDescent="0.2">
@@ -1183,10 +1192,10 @@
         <v>6</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
@@ -1197,10 +1206,10 @@
         <v>6</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1211,7 +1220,7 @@
         <v>6</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1222,10 +1231,10 @@
         <v>6</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1236,7 +1245,7 @@
         <v>6</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
@@ -1247,10 +1256,10 @@
         <v>6</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1261,18 +1270,18 @@
         <v>6</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="16" hidden="1" x14ac:dyDescent="0.2">
@@ -1283,7 +1292,7 @@
         <v>6</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1302,16 +1311,16 @@
     </row>
     <row r="43" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B43" t="s">
         <v>7</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
@@ -1322,10 +1331,10 @@
         <v>7</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
@@ -1336,10 +1345,10 @@
         <v>7</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1350,7 +1359,7 @@
         <v>7</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
@@ -1361,7 +1370,7 @@
         <v>7</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>48</v>
@@ -1375,10 +1384,10 @@
         <v>7</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="112" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>25</v>
       </c>
@@ -1386,10 +1395,10 @@
         <v>6</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="112" x14ac:dyDescent="0.2">
@@ -1400,10 +1409,10 @@
         <v>7</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1414,18 +1423,18 @@
         <v>7</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B52" t="s">
         <v>7</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="256" hidden="1" x14ac:dyDescent="0.2">
@@ -1436,10 +1445,10 @@
         <v>8</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1453,21 +1462,21 @@
         <v>41</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B55" t="s">
         <v>8</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
@@ -1478,10 +1487,10 @@
         <v>8</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1492,7 +1501,7 @@
         <v>8</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1503,7 +1512,7 @@
         <v>8</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
@@ -1514,7 +1523,7 @@
         <v>8</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>49</v>
@@ -1528,18 +1537,18 @@
         <v>8</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B61" t="s">
         <v>8</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="16" hidden="1" x14ac:dyDescent="0.2">
@@ -1550,7 +1559,7 @@
         <v>8</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1561,10 +1570,10 @@
         <v>29</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1575,10 +1584,10 @@
         <v>29</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
@@ -1592,7 +1601,7 @@
         <v>41</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1603,10 +1612,10 @@
         <v>29</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1617,7 +1626,7 @@
         <v>4</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1628,7 +1637,7 @@
         <v>4</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
@@ -1639,544 +1648,547 @@
         <v>4</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="144" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>19</v>
       </c>
       <c r="B70" t="s">
-        <v>4</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>55</v>
+        <v>8</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
       </c>
-      <c r="C72" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>53</v>
+      <c r="C72" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
-      <c r="C73" s="5" t="s">
-        <v>86</v>
+      <c r="C73" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
       </c>
-      <c r="C74" s="4" t="s">
-        <v>41</v>
+      <c r="C74" s="5" t="s">
+        <v>85</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="128" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="B75" t="s">
+        <v>8</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>25</v>
+      </c>
+      <c r="B76" t="s">
         <v>4</v>
       </c>
-      <c r="C75" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>3</v>
-      </c>
-      <c r="B76" t="s">
-        <v>9</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>55</v>
+      <c r="C76" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="B77" t="s">
-        <v>9</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>55</v>
+        <v>4</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
       </c>
-      <c r="C78" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>84</v>
+      <c r="C78" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>55</v>
+      <c r="C80" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B82" t="s">
         <v>9</v>
       </c>
-      <c r="C82" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="C82" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
       </c>
-      <c r="C83" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="272" hidden="1" x14ac:dyDescent="0.2">
+      <c r="C83" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
+        <v>26</v>
+      </c>
+      <c r="B84" t="s">
+        <v>9</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>42</v>
+      </c>
+      <c r="B85" t="s">
+        <v>9</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="272" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
         <v>3</v>
-      </c>
-      <c r="B84" t="s">
-        <v>10</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>69</v>
-      </c>
-      <c r="B85" t="s">
-        <v>10</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>81</v>
       </c>
       <c r="B86" t="s">
         <v>10</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="B87" t="s">
         <v>10</v>
       </c>
       <c r="C87" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D87" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D87" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="88" spans="1:4" ht="160" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>19</v>
+        <v>80</v>
       </c>
       <c r="B88" t="s">
         <v>10</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
         <v>10</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B90" t="s">
         <v>10</v>
       </c>
-      <c r="C90" s="1" t="s">
-        <v>55</v>
+      <c r="C90" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B91" t="s">
         <v>10</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B92" t="s">
         <v>10</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B93" t="s">
         <v>10</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B94" t="s">
         <v>10</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="128" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="B95" t="s">
         <v>10</v>
       </c>
-      <c r="C95" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
+      <c r="C95" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B96" t="s">
         <v>10</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D96" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
+        <v>67</v>
+      </c>
+      <c r="B97" t="s">
+        <v>10</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>38</v>
+      </c>
+      <c r="B98" t="s">
+        <v>10</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
         <v>16</v>
-      </c>
-      <c r="B97" t="s">
-        <v>17</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>37</v>
-      </c>
-      <c r="B98" t="s">
-        <v>17</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>31</v>
       </c>
       <c r="B99" t="s">
         <v>17</v>
       </c>
-      <c r="C99" s="1" t="s">
-        <v>55</v>
+      <c r="C99" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D99" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>37</v>
+      </c>
+      <c r="B100" t="s">
+        <v>17</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row r="101" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>31</v>
+      </c>
+      <c r="B101" t="s">
+        <v>17</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>16</v>
-      </c>
-      <c r="B100" t="s">
-        <v>18</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>22</v>
-      </c>
-      <c r="B101" t="s">
-        <v>18</v>
-      </c>
-      <c r="C101" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D101" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>31</v>
       </c>
       <c r="B102" t="s">
         <v>18</v>
       </c>
-      <c r="C102" s="1" t="s">
+      <c r="C102" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D102" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D102" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+    </row>
+    <row r="103" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B103" t="s">
         <v>18</v>
       </c>
-      <c r="C103" s="5" t="s">
-        <v>86</v>
+      <c r="C103" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>109</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
+        <v>31</v>
+      </c>
+      <c r="B104" t="s">
+        <v>18</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>25</v>
+      </c>
+      <c r="B105" t="s">
+        <v>18</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>3</v>
-      </c>
-      <c r="B104" t="s">
-        <v>11</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>19</v>
-      </c>
-      <c r="B105" t="s">
-        <v>11</v>
-      </c>
-      <c r="C105" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="112" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>25</v>
       </c>
       <c r="B106" t="s">
         <v>11</v>
       </c>
-      <c r="C106" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>62</v>
+      <c r="C106" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="B107" t="s">
         <v>11</v>
       </c>
-      <c r="C107" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
+      <c r="C107" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="112" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B108" t="s">
         <v>11</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="B109" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="112" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="B110" t="s">
-        <v>13</v>
-      </c>
-      <c r="C110" s="4" t="s">
-        <v>41</v>
+        <v>11</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>85</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="B111" t="s">
         <v>13</v>
@@ -2187,7 +2199,7 @@
     </row>
     <row r="112" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="B112" t="s">
         <v>13</v>
@@ -2196,35 +2208,60 @@
         <v>41</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B113" t="s">
         <v>13</v>
       </c>
-      <c r="C113" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D113" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C117" s="5"/>
+      <c r="C113" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>22</v>
+      </c>
+      <c r="B114" t="s">
+        <v>13</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>46</v>
+      </c>
+      <c r="B115" t="s">
+        <v>13</v>
+      </c>
+      <c r="C115" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C119" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D113" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:D115" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
         <filter val="MEX"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D113">
-      <sortCondition ref="B1:B113"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D115">
+      <sortCondition ref="B1:B115"/>
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C37">

</xml_diff>